<commit_message>
20260208 pushed work from Friday
</commit_message>
<xml_diff>
--- a/2026_Brightspace/timetable_2026-02-06.xlsx
+++ b/2026_Brightspace/timetable_2026-02-06.xlsx
@@ -11,6 +11,9 @@
     <sheet name="Activities" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Activities_time_table" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
+  <definedNames>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Activities!$A$1:$F$85</definedName>
+  </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -21,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1035" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1033" uniqueCount="108">
   <si>
     <t xml:space="preserve">Chemistry for Earth Sciences</t>
   </si>
@@ -119,25 +122,19 @@
     <t xml:space="preserve">Week 3.6 (16 March 2026 - 22 March 2026)</t>
   </si>
   <si>
+    <t xml:space="preserve">Aqueous geochemistry examples</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Week 3.7 (23 March 2026 - 29 March 2026)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Atmospheric examples</t>
   </si>
   <si>
-    <t xml:space="preserve">Week 3.7 (23 March 2026 - 29 March 2026)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aqueous geochemistry examples</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Solids Pourbaix diagrams</t>
-  </si>
-  <si>
     <t xml:space="preserve">Week 3.8 (30 March 2026 - 5 April 2026)</t>
   </si>
   <si>
     <t xml:space="preserve">Solids, Pourbaix diagrams</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aqueous geochemstry examples…</t>
   </si>
   <si>
     <t xml:space="preserve">Week 3.9 (6 April 2026 - 12 April 2026)</t>
@@ -758,7 +755,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:F85"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -1108,7 +1105,7 @@
         <v>20</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E37" s="12" t="s">
         <v>21</v>
@@ -1128,11 +1125,12 @@
         <v>20</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E38" s="12" t="s">
         <v>21</v>
       </c>
+      <c r="F38" s="0"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="5" t="s">
@@ -1150,7 +1148,7 @@
         <v>20</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E41" s="12" t="s">
         <v>21</v>
@@ -1170,18 +1168,16 @@
         <v>20</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E42" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="F42" s="1" t="s">
-        <v>35</v>
-      </c>
+      <c r="F42" s="0"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1201,7 +1197,7 @@
         <v>21</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1220,13 +1216,10 @@
       <c r="E46" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="F46" s="1" t="s">
-        <v>38</v>
-      </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="13" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B48" s="14"/>
       <c r="C48" s="15"/>
@@ -1242,21 +1235,21 @@
         <v>0.0833333333333333</v>
       </c>
       <c r="C49" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="D49" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="E49" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="D49" s="19" t="s">
+      <c r="F49" s="14" t="s">
         <v>41</v>
-      </c>
-      <c r="E49" s="20" t="s">
-        <v>42</v>
-      </c>
-      <c r="F49" s="14" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1273,10 +1266,10 @@
         <v>8</v>
       </c>
       <c r="E52" s="12" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1293,12 +1286,12 @@
         <v>8</v>
       </c>
       <c r="E53" s="12" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1315,10 +1308,10 @@
         <v>12</v>
       </c>
       <c r="E56" s="12" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1333,7 +1326,7 @@
       </c>
       <c r="D57" s="5"/>
       <c r="E57" s="12" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1350,12 +1343,12 @@
         <v>12</v>
       </c>
       <c r="E58" s="12" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="5" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1372,10 +1365,10 @@
         <v>10</v>
       </c>
       <c r="E61" s="12" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1390,29 +1383,29 @@
       </c>
       <c r="D62" s="12"/>
       <c r="E62" s="12" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B65" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C65" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="B65" s="5" t="s">
+      <c r="D65" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="C65" s="8" t="s">
+      <c r="E65" s="5" t="s">
         <v>55</v>
-      </c>
-      <c r="D65" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="E65" s="5" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1432,7 +1425,7 @@
         <v>21</v>
       </c>
       <c r="F66" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1446,10 +1439,10 @@
         <v>6</v>
       </c>
       <c r="D67" s="3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E67" s="12" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1460,18 +1453,18 @@
         <v>0.166666666666667</v>
       </c>
       <c r="C68" s="11" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D68" s="3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E68" s="12" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="5" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1482,16 +1475,16 @@
         <v>0.166666666666667</v>
       </c>
       <c r="C71" s="11" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D71" s="3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E71" s="12" t="s">
         <v>21</v>
       </c>
       <c r="F71" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1502,10 +1495,10 @@
         <v>0.166666666666667</v>
       </c>
       <c r="C72" s="11" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D72" s="3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E72" s="12" t="s">
         <v>21</v>
@@ -1513,7 +1506,7 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="5" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1524,16 +1517,16 @@
         <v>0.166666666666667</v>
       </c>
       <c r="C75" s="11" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D75" s="3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E75" s="12" t="s">
         <v>21</v>
       </c>
       <c r="F75" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1544,10 +1537,10 @@
         <v>0.166666666666667</v>
       </c>
       <c r="C76" s="11" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D76" s="3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E76" s="12" t="s">
         <v>21</v>
@@ -1555,7 +1548,7 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="13" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B78" s="14"/>
       <c r="C78" s="15"/>
@@ -1571,21 +1564,21 @@
         <v>0.125</v>
       </c>
       <c r="C79" s="18" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D79" s="19" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E79" s="20" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="F79" s="14" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="21" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B81" s="22"/>
       <c r="C81" s="23"/>
@@ -1601,21 +1594,21 @@
         <v>0.0833333333333333</v>
       </c>
       <c r="C82" s="26" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D82" s="27" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E82" s="28" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="F82" s="22" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="13" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B84" s="14"/>
       <c r="C84" s="15"/>
@@ -1631,16 +1624,16 @@
         <v>0.125</v>
       </c>
       <c r="C85" s="18" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D85" s="19" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E85" s="20" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F85" s="14" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -1651,7 +1644,7 @@
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -1677,63 +1670,63 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B2" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="C2" s="5" t="s">
+      <c r="E2" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="F2" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="E2" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>57</v>
-      </c>
       <c r="G2" s="5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H2" s="5" t="s">
         <v>16</v>
       </c>
       <c r="I2" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="K2" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="J2" s="5" t="s">
+      <c r="L2" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="K2" s="5" t="s">
+      <c r="M2" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="L2" s="5" t="s">
+      <c r="N2" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="M2" s="5" t="s">
+      <c r="O2" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="N2" s="5" t="s">
+      <c r="P2" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="O2" s="5" t="s">
+      <c r="Q2" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="P2" s="5" t="s">
+      <c r="R2" s="5" t="s">
         <v>83</v>
-      </c>
-      <c r="Q2" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="R2" s="5" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1760,16 +1753,16 @@
         <v>20</v>
       </c>
       <c r="I3" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J3" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K3" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L3" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N3" s="12"/>
       <c r="O3" s="1" t="b">
@@ -1813,16 +1806,16 @@
         <v>5</v>
       </c>
       <c r="I4" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J4" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K4" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L4" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N4" s="12"/>
       <c r="O4" s="1" t="b">
@@ -1866,16 +1859,16 @@
         <v>6</v>
       </c>
       <c r="I5" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J5" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K5" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L5" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N5" s="12"/>
       <c r="O5" s="1" t="b">
@@ -1919,16 +1912,16 @@
         <v>20</v>
       </c>
       <c r="I6" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J6" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K6" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L6" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N6" s="12"/>
       <c r="O6" s="1" t="b">
@@ -1972,16 +1965,16 @@
         <v>5</v>
       </c>
       <c r="I7" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J7" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K7" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L7" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N7" s="12"/>
       <c r="O7" s="1" t="b">
@@ -2025,16 +2018,16 @@
         <v>6</v>
       </c>
       <c r="I8" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J8" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K8" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L8" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N8" s="12"/>
       <c r="O8" s="1" t="b">
@@ -2056,63 +2049,63 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D11" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B11" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="C11" s="5" t="s">
+      <c r="E11" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="F11" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="E11" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>57</v>
-      </c>
       <c r="G11" s="5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H11" s="5" t="s">
         <v>16</v>
       </c>
       <c r="I11" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="J11" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="K11" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="J11" s="5" t="s">
+      <c r="L11" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="K11" s="5" t="s">
+      <c r="M11" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="L11" s="5" t="s">
+      <c r="N11" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="M11" s="5" t="s">
+      <c r="O11" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="N11" s="5" t="s">
+      <c r="P11" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="O11" s="5" t="s">
+      <c r="Q11" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="P11" s="5" t="s">
+      <c r="R11" s="5" t="s">
         <v>83</v>
-      </c>
-      <c r="Q11" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="R11" s="5" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2139,16 +2132,16 @@
         <v>20</v>
       </c>
       <c r="I12" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J12" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K12" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L12" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N12" s="12"/>
       <c r="O12" s="1" t="b">
@@ -2192,16 +2185,16 @@
         <v>5</v>
       </c>
       <c r="I13" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J13" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K13" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L13" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N13" s="12"/>
       <c r="O13" s="1" t="b">
@@ -2245,16 +2238,16 @@
         <v>6</v>
       </c>
       <c r="I14" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J14" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K14" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L14" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N14" s="12"/>
       <c r="O14" s="1" t="b">
@@ -2298,16 +2291,16 @@
         <v>20</v>
       </c>
       <c r="I15" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J15" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K15" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L15" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N15" s="12"/>
       <c r="O15" s="1" t="b">
@@ -2351,16 +2344,16 @@
         <v>5</v>
       </c>
       <c r="I16" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J16" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K16" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L16" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N16" s="12"/>
       <c r="O16" s="1" t="b">
@@ -2404,16 +2397,16 @@
         <v>6</v>
       </c>
       <c r="I17" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J17" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K17" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L17" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N17" s="12"/>
       <c r="O17" s="1" t="b">
@@ -2435,63 +2428,63 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D20" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B20" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="C20" s="5" t="s">
+      <c r="E20" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D20" s="5" t="s">
+      <c r="F20" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="E20" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="F20" s="5" t="s">
-        <v>57</v>
-      </c>
       <c r="G20" s="5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H20" s="5" t="s">
         <v>16</v>
       </c>
       <c r="I20" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="J20" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="K20" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="J20" s="5" t="s">
+      <c r="L20" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="K20" s="5" t="s">
+      <c r="M20" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="L20" s="5" t="s">
+      <c r="N20" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="M20" s="5" t="s">
+      <c r="O20" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="N20" s="5" t="s">
+      <c r="P20" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="O20" s="5" t="s">
+      <c r="Q20" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="P20" s="5" t="s">
+      <c r="R20" s="5" t="s">
         <v>83</v>
-      </c>
-      <c r="Q20" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="R20" s="5" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2518,16 +2511,16 @@
         <v>20</v>
       </c>
       <c r="I21" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J21" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K21" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L21" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N21" s="12"/>
       <c r="O21" s="1" t="b">
@@ -2571,16 +2564,16 @@
         <v>5</v>
       </c>
       <c r="I22" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J22" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K22" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L22" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N22" s="12"/>
       <c r="O22" s="1" t="b">
@@ -2624,16 +2617,16 @@
         <v>6</v>
       </c>
       <c r="I23" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J23" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K23" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L23" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N23" s="12"/>
       <c r="O23" s="1" t="b">
@@ -2677,16 +2670,16 @@
         <v>20</v>
       </c>
       <c r="I24" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J24" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K24" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L24" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N24" s="12"/>
       <c r="O24" s="1" t="b">
@@ -2730,16 +2723,16 @@
         <v>5</v>
       </c>
       <c r="I25" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J25" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K25" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L25" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N25" s="12"/>
       <c r="O25" s="1" t="b">
@@ -2783,16 +2776,16 @@
         <v>6</v>
       </c>
       <c r="I26" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J26" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K26" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L26" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N26" s="12"/>
       <c r="O26" s="1" t="b">
@@ -2814,63 +2807,63 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D29" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B29" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="C29" s="5" t="s">
+      <c r="E29" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D29" s="5" t="s">
+      <c r="F29" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="E29" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="F29" s="5" t="s">
-        <v>57</v>
-      </c>
       <c r="G29" s="5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H29" s="5" t="s">
         <v>16</v>
       </c>
       <c r="I29" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="J29" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="K29" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="J29" s="5" t="s">
+      <c r="L29" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="K29" s="5" t="s">
+      <c r="M29" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="L29" s="5" t="s">
+      <c r="N29" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="M29" s="5" t="s">
+      <c r="O29" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="N29" s="5" t="s">
+      <c r="P29" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="O29" s="5" t="s">
+      <c r="Q29" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="P29" s="5" t="s">
+      <c r="R29" s="5" t="s">
         <v>83</v>
-      </c>
-      <c r="Q29" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="R29" s="5" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2897,16 +2890,16 @@
         <v>20</v>
       </c>
       <c r="I30" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J30" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K30" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L30" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N30" s="12"/>
       <c r="O30" s="1" t="b">
@@ -2950,16 +2943,16 @@
         <v>5</v>
       </c>
       <c r="I31" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K31" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L31" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N31" s="12"/>
       <c r="O31" s="1" t="b">
@@ -3003,16 +2996,16 @@
         <v>6</v>
       </c>
       <c r="I32" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J32" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K32" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L32" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N32" s="12"/>
       <c r="O32" s="1" t="b">
@@ -3056,16 +3049,16 @@
         <v>20</v>
       </c>
       <c r="I33" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J33" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K33" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L33" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N33" s="12"/>
       <c r="O33" s="1" t="b">
@@ -3109,16 +3102,16 @@
         <v>5</v>
       </c>
       <c r="I34" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J34" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K34" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L34" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N34" s="12"/>
       <c r="O34" s="1" t="b">
@@ -3162,16 +3155,16 @@
         <v>6</v>
       </c>
       <c r="I35" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J35" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K35" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L35" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N35" s="12"/>
       <c r="O35" s="1" t="b">
@@ -3193,63 +3186,63 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C38" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D38" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B38" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="C38" s="5" t="s">
+      <c r="E38" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D38" s="5" t="s">
+      <c r="F38" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="E38" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="F38" s="5" t="s">
-        <v>57</v>
-      </c>
       <c r="G38" s="5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H38" s="5" t="s">
         <v>16</v>
       </c>
       <c r="I38" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="J38" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="K38" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="J38" s="5" t="s">
+      <c r="L38" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="K38" s="5" t="s">
+      <c r="M38" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="L38" s="5" t="s">
+      <c r="N38" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="M38" s="5" t="s">
+      <c r="O38" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="N38" s="5" t="s">
+      <c r="P38" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="O38" s="5" t="s">
+      <c r="Q38" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="P38" s="5" t="s">
+      <c r="R38" s="5" t="s">
         <v>83</v>
-      </c>
-      <c r="Q38" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="R38" s="5" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3276,16 +3269,16 @@
         <v>20</v>
       </c>
       <c r="I39" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J39" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K39" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L39" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N39" s="12"/>
       <c r="O39" s="1" t="b">
@@ -3329,16 +3322,16 @@
         <v>5</v>
       </c>
       <c r="I40" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J40" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K40" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L40" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N40" s="12"/>
       <c r="O40" s="1" t="b">
@@ -3382,16 +3375,16 @@
         <v>6</v>
       </c>
       <c r="I41" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J41" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K41" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L41" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N41" s="12"/>
       <c r="O41" s="1" t="b">
@@ -3435,16 +3428,16 @@
         <v>20</v>
       </c>
       <c r="I42" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J42" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K42" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L42" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N42" s="12"/>
       <c r="O42" s="1" t="b">
@@ -3488,16 +3481,16 @@
         <v>5</v>
       </c>
       <c r="I43" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J43" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K43" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L43" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N43" s="12"/>
       <c r="O43" s="1" t="b">
@@ -3541,16 +3534,16 @@
         <v>6</v>
       </c>
       <c r="I44" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J44" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K44" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L44" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N44" s="12"/>
       <c r="O44" s="1" t="b">
@@ -3572,63 +3565,63 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B47" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C47" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D47" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B47" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="C47" s="5" t="s">
+      <c r="E47" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D47" s="5" t="s">
+      <c r="F47" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="E47" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="F47" s="5" t="s">
-        <v>57</v>
-      </c>
       <c r="G47" s="5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H47" s="5" t="s">
         <v>16</v>
       </c>
       <c r="I47" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="J47" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="K47" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="J47" s="5" t="s">
+      <c r="L47" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="K47" s="5" t="s">
+      <c r="M47" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="L47" s="5" t="s">
+      <c r="N47" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="M47" s="5" t="s">
+      <c r="O47" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="N47" s="5" t="s">
+      <c r="P47" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="O47" s="5" t="s">
+      <c r="Q47" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="P47" s="5" t="s">
+      <c r="R47" s="5" t="s">
         <v>83</v>
-      </c>
-      <c r="Q47" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="R47" s="5" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3655,16 +3648,16 @@
         <v>20</v>
       </c>
       <c r="I48" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J48" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K48" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L48" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N48" s="12"/>
       <c r="O48" s="1" t="b">
@@ -3708,16 +3701,16 @@
         <v>5</v>
       </c>
       <c r="I49" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J49" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K49" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L49" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N49" s="12"/>
       <c r="O49" s="1" t="b">
@@ -3761,16 +3754,16 @@
         <v>6</v>
       </c>
       <c r="I50" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J50" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K50" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L50" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N50" s="12"/>
       <c r="O50" s="1" t="b">
@@ -3814,16 +3807,16 @@
         <v>20</v>
       </c>
       <c r="I51" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J51" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K51" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L51" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N51" s="12"/>
       <c r="O51" s="1" t="b">
@@ -3867,16 +3860,16 @@
         <v>5</v>
       </c>
       <c r="I52" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J52" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K52" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L52" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N52" s="12"/>
       <c r="O52" s="1" t="b">
@@ -3920,16 +3913,16 @@
         <v>6</v>
       </c>
       <c r="I53" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J53" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K53" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L53" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N53" s="12"/>
       <c r="O53" s="1" t="b">
@@ -3951,63 +3944,63 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="5" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B56" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C56" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D56" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B56" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="C56" s="5" t="s">
+      <c r="E56" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D56" s="5" t="s">
+      <c r="F56" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="E56" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="F56" s="5" t="s">
-        <v>57</v>
-      </c>
       <c r="G56" s="5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H56" s="5" t="s">
         <v>16</v>
       </c>
       <c r="I56" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="J56" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="K56" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="J56" s="5" t="s">
+      <c r="L56" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="K56" s="5" t="s">
+      <c r="M56" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="L56" s="5" t="s">
+      <c r="N56" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="M56" s="5" t="s">
+      <c r="O56" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="N56" s="5" t="s">
+      <c r="P56" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="O56" s="5" t="s">
+      <c r="Q56" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="P56" s="5" t="s">
+      <c r="R56" s="5" t="s">
         <v>83</v>
-      </c>
-      <c r="Q56" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="R56" s="5" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4034,16 +4027,16 @@
         <v>20</v>
       </c>
       <c r="I57" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J57" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K57" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L57" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N57" s="12"/>
       <c r="O57" s="1" t="b">
@@ -4087,16 +4080,16 @@
         <v>5</v>
       </c>
       <c r="I58" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J58" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K58" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L58" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N58" s="12"/>
       <c r="O58" s="1" t="b">
@@ -4140,16 +4133,16 @@
         <v>6</v>
       </c>
       <c r="I59" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J59" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K59" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L59" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N59" s="12"/>
       <c r="O59" s="1" t="b">
@@ -4193,16 +4186,16 @@
         <v>20</v>
       </c>
       <c r="I60" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J60" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K60" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L60" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N60" s="12"/>
       <c r="O60" s="1" t="b">
@@ -4246,16 +4239,16 @@
         <v>5</v>
       </c>
       <c r="I61" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J61" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K61" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L61" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N61" s="12"/>
       <c r="O61" s="1" t="b">
@@ -4299,16 +4292,16 @@
         <v>6</v>
       </c>
       <c r="I62" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J62" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K62" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L62" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N62" s="12"/>
       <c r="O62" s="1" t="b">
@@ -4330,63 +4323,63 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="5" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B65" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C65" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D65" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B65" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="C65" s="5" t="s">
+      <c r="E65" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D65" s="5" t="s">
+      <c r="F65" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="E65" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="F65" s="5" t="s">
-        <v>57</v>
-      </c>
       <c r="G65" s="5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H65" s="5" t="s">
         <v>16</v>
       </c>
       <c r="I65" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="J65" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="K65" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="J65" s="5" t="s">
+      <c r="L65" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="K65" s="5" t="s">
+      <c r="M65" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="L65" s="5" t="s">
+      <c r="N65" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="M65" s="5" t="s">
+      <c r="O65" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="N65" s="5" t="s">
+      <c r="P65" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="O65" s="5" t="s">
+      <c r="Q65" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="P65" s="5" t="s">
+      <c r="R65" s="5" t="s">
         <v>83</v>
-      </c>
-      <c r="Q65" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="R65" s="5" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4413,16 +4406,16 @@
         <v>20</v>
       </c>
       <c r="I66" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J66" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K66" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L66" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N66" s="12"/>
       <c r="O66" s="1" t="b">
@@ -4466,16 +4459,16 @@
         <v>5</v>
       </c>
       <c r="I67" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J67" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K67" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L67" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N67" s="12"/>
       <c r="O67" s="1" t="b">
@@ -4519,16 +4512,16 @@
         <v>6</v>
       </c>
       <c r="I68" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J68" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K68" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L68" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N68" s="12"/>
       <c r="O68" s="1" t="b">
@@ -4572,16 +4565,16 @@
         <v>20</v>
       </c>
       <c r="I69" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J69" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K69" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L69" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N69" s="12"/>
       <c r="O69" s="1" t="b">
@@ -4625,16 +4618,16 @@
         <v>5</v>
       </c>
       <c r="I70" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J70" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K70" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L70" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N70" s="12"/>
       <c r="O70" s="1" t="b">
@@ -4678,16 +4671,16 @@
         <v>6</v>
       </c>
       <c r="I71" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J71" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K71" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L71" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N71" s="12"/>
       <c r="O71" s="1" t="b">
@@ -4709,68 +4702,68 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="5" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B74" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C74" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D74" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B74" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="C74" s="5" t="s">
+      <c r="E74" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D74" s="5" t="s">
+      <c r="F74" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="E74" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="F74" s="5" t="s">
-        <v>57</v>
-      </c>
       <c r="G74" s="5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H74" s="5" t="s">
         <v>16</v>
       </c>
       <c r="I74" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="J74" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="K74" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="J74" s="5" t="s">
+      <c r="L74" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="K74" s="5" t="s">
+      <c r="M74" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="L74" s="5" t="s">
+      <c r="N74" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="M74" s="5" t="s">
+      <c r="O74" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="N74" s="5" t="s">
+      <c r="P74" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="O74" s="5" t="s">
+      <c r="Q74" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="P74" s="5" t="s">
+      <c r="R74" s="5" t="s">
         <v>83</v>
-      </c>
-      <c r="Q74" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="R74" s="5" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="12" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B75" s="12" t="s">
         <v>1</v>
@@ -4789,22 +4782,22 @@
         <v>0.0833333333333333</v>
       </c>
       <c r="H75" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="I75" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="J75" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="I75" s="12" t="s">
-        <v>86</v>
-      </c>
-      <c r="J75" s="12" t="s">
-        <v>42</v>
-      </c>
       <c r="K75" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L75" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N75" s="12" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="O75" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -4825,63 +4818,63 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="5" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B78" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C78" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D78" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B78" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="C78" s="5" t="s">
+      <c r="E78" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D78" s="5" t="s">
+      <c r="F78" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="E78" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="F78" s="5" t="s">
-        <v>57</v>
-      </c>
       <c r="G78" s="5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H78" s="5" t="s">
         <v>16</v>
       </c>
       <c r="I78" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="J78" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="K78" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="J78" s="5" t="s">
+      <c r="L78" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="K78" s="5" t="s">
+      <c r="M78" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="L78" s="5" t="s">
+      <c r="N78" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="M78" s="5" t="s">
+      <c r="O78" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="N78" s="5" t="s">
+      <c r="P78" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="O78" s="5" t="s">
+      <c r="Q78" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="P78" s="5" t="s">
+      <c r="R78" s="5" t="s">
         <v>83</v>
-      </c>
-      <c r="Q78" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="R78" s="5" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4908,16 +4901,16 @@
         <v>20</v>
       </c>
       <c r="I79" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J79" s="12" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="K79" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L79" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N79" s="12"/>
       <c r="O79" s="1" t="b">
@@ -4961,16 +4954,16 @@
         <v>5</v>
       </c>
       <c r="I80" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J80" s="12" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="K80" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L80" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N80" s="12"/>
       <c r="O80" s="1" t="b">
@@ -5014,16 +5007,16 @@
         <v>6</v>
       </c>
       <c r="I81" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J81" s="12" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="K81" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L81" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N81" s="12"/>
       <c r="O81" s="1" t="b">
@@ -5067,16 +5060,16 @@
         <v>20</v>
       </c>
       <c r="I82" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J82" s="12" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="K82" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L82" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N82" s="12"/>
       <c r="O82" s="1" t="b">
@@ -5120,16 +5113,16 @@
         <v>5</v>
       </c>
       <c r="I83" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J83" s="12" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="K83" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L83" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N83" s="12"/>
       <c r="O83" s="1" t="b">
@@ -5173,16 +5166,16 @@
         <v>6</v>
       </c>
       <c r="I84" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J84" s="12" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="K84" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L84" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N84" s="12"/>
       <c r="O84" s="1" t="b">
@@ -5204,63 +5197,63 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="5" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B87" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C87" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D87" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B87" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="C87" s="5" t="s">
+      <c r="E87" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D87" s="5" t="s">
+      <c r="F87" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="E87" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="F87" s="5" t="s">
-        <v>57</v>
-      </c>
       <c r="G87" s="5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H87" s="5" t="s">
         <v>16</v>
       </c>
       <c r="I87" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="J87" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="K87" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="J87" s="5" t="s">
+      <c r="L87" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="K87" s="5" t="s">
+      <c r="M87" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="L87" s="5" t="s">
+      <c r="N87" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="M87" s="5" t="s">
+      <c r="O87" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="N87" s="5" t="s">
+      <c r="P87" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="O87" s="5" t="s">
+      <c r="Q87" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="P87" s="5" t="s">
+      <c r="R87" s="5" t="s">
         <v>83</v>
-      </c>
-      <c r="Q87" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="R87" s="5" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5287,16 +5280,16 @@
         <v>20</v>
       </c>
       <c r="I88" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J88" s="12" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="K88" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L88" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N88" s="12"/>
       <c r="O88" s="1" t="b">
@@ -5340,16 +5333,16 @@
         <v>5</v>
       </c>
       <c r="I89" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J89" s="12" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="K89" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L89" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N89" s="12"/>
       <c r="O89" s="1" t="b">
@@ -5393,16 +5386,16 @@
         <v>6</v>
       </c>
       <c r="I90" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J90" s="12" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="K90" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L90" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N90" s="12"/>
       <c r="O90" s="1" t="b">
@@ -5446,16 +5439,16 @@
         <v>20</v>
       </c>
       <c r="I91" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J91" s="12" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="K91" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L91" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N91" s="12"/>
       <c r="O91" s="1" t="b">
@@ -5499,16 +5492,16 @@
         <v>5</v>
       </c>
       <c r="I92" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J92" s="12" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="K92" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L92" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N92" s="12"/>
       <c r="O92" s="1" t="b">
@@ -5552,16 +5545,16 @@
         <v>6</v>
       </c>
       <c r="I93" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J93" s="12" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="K93" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L93" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N93" s="12"/>
       <c r="O93" s="1" t="b">
@@ -5583,63 +5576,63 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="5" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B96" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C96" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D96" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B96" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="C96" s="5" t="s">
+      <c r="E96" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D96" s="5" t="s">
+      <c r="F96" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="E96" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="F96" s="5" t="s">
-        <v>57</v>
-      </c>
       <c r="G96" s="5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H96" s="5" t="s">
         <v>16</v>
       </c>
       <c r="I96" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="J96" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="K96" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="J96" s="5" t="s">
+      <c r="L96" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="K96" s="5" t="s">
+      <c r="M96" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="L96" s="5" t="s">
+      <c r="N96" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="M96" s="5" t="s">
+      <c r="O96" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="N96" s="5" t="s">
+      <c r="P96" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="O96" s="5" t="s">
+      <c r="Q96" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="P96" s="5" t="s">
+      <c r="R96" s="5" t="s">
         <v>83</v>
-      </c>
-      <c r="Q96" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="R96" s="5" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5666,16 +5659,16 @@
         <v>20</v>
       </c>
       <c r="I97" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J97" s="12" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="K97" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L97" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N97" s="12"/>
       <c r="O97" s="1" t="b">
@@ -5719,16 +5712,16 @@
         <v>5</v>
       </c>
       <c r="I98" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J98" s="12" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="K98" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L98" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N98" s="12"/>
       <c r="O98" s="1" t="b">
@@ -5772,16 +5765,16 @@
         <v>6</v>
       </c>
       <c r="I99" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J99" s="12" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="K99" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L99" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N99" s="12"/>
       <c r="O99" s="1" t="b">
@@ -5803,63 +5796,63 @@
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="5" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B102" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C102" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D102" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B102" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="C102" s="5" t="s">
+      <c r="E102" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D102" s="5" t="s">
+      <c r="F102" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="E102" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="F102" s="5" t="s">
-        <v>57</v>
-      </c>
       <c r="G102" s="5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H102" s="5" t="s">
         <v>16</v>
       </c>
       <c r="I102" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="J102" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="K102" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="J102" s="5" t="s">
+      <c r="L102" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="K102" s="5" t="s">
+      <c r="M102" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="L102" s="5" t="s">
+      <c r="N102" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="M102" s="5" t="s">
+      <c r="O102" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="N102" s="5" t="s">
+      <c r="P102" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="O102" s="5" t="s">
+      <c r="Q102" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="P102" s="5" t="s">
+      <c r="R102" s="5" t="s">
         <v>83</v>
-      </c>
-      <c r="Q102" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="R102" s="5" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5886,16 +5879,16 @@
         <v>20</v>
       </c>
       <c r="I103" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J103" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K103" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L103" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N103" s="12"/>
       <c r="O103" s="1" t="b">
@@ -5939,16 +5932,16 @@
         <v>5</v>
       </c>
       <c r="I104" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J104" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K104" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L104" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N104" s="12"/>
       <c r="O104" s="1" t="b">
@@ -5992,16 +5985,16 @@
         <v>6</v>
       </c>
       <c r="I105" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J105" s="12" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="K105" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L105" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N105" s="12"/>
       <c r="O105" s="1" t="b">
@@ -6042,19 +6035,19 @@
         <v>0.166666666666667</v>
       </c>
       <c r="H106" s="12" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="I106" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J106" s="12" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="K106" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L106" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N106" s="12"/>
       <c r="O106" s="1" t="b">
@@ -6076,63 +6069,63 @@
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="5" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B109" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C109" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D109" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B109" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="C109" s="5" t="s">
+      <c r="E109" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D109" s="5" t="s">
+      <c r="F109" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="E109" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="F109" s="5" t="s">
-        <v>57</v>
-      </c>
       <c r="G109" s="5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H109" s="5" t="s">
         <v>16</v>
       </c>
       <c r="I109" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="J109" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="K109" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="J109" s="5" t="s">
+      <c r="L109" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="K109" s="5" t="s">
+      <c r="M109" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="L109" s="5" t="s">
+      <c r="N109" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="M109" s="5" t="s">
+      <c r="O109" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="N109" s="5" t="s">
+      <c r="P109" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="O109" s="5" t="s">
+      <c r="Q109" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="P109" s="5" t="s">
+      <c r="R109" s="5" t="s">
         <v>83</v>
-      </c>
-      <c r="Q109" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="R109" s="5" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6156,19 +6149,19 @@
         <v>0.166666666666667</v>
       </c>
       <c r="H110" s="12" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I110" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J110" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K110" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L110" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N110" s="12"/>
       <c r="O110" s="1" t="b">
@@ -6209,19 +6202,19 @@
         <v>0.166666666666667</v>
       </c>
       <c r="H111" s="12" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I111" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J111" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K111" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L111" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N111" s="12"/>
       <c r="O111" s="1" t="b">
@@ -6243,63 +6236,63 @@
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="5" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B114" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C114" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D114" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B114" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="C114" s="5" t="s">
+      <c r="E114" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D114" s="5" t="s">
+      <c r="F114" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="E114" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="F114" s="5" t="s">
-        <v>57</v>
-      </c>
       <c r="G114" s="5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H114" s="5" t="s">
         <v>16</v>
       </c>
       <c r="I114" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="J114" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="K114" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="J114" s="5" t="s">
+      <c r="L114" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="K114" s="5" t="s">
+      <c r="M114" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="L114" s="5" t="s">
+      <c r="N114" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="M114" s="5" t="s">
+      <c r="O114" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="N114" s="5" t="s">
+      <c r="P114" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="O114" s="5" t="s">
+      <c r="Q114" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="P114" s="5" t="s">
+      <c r="R114" s="5" t="s">
         <v>83</v>
-      </c>
-      <c r="Q114" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="R114" s="5" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6323,19 +6316,19 @@
         <v>0.166666666666667</v>
       </c>
       <c r="H115" s="12" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I115" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J115" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K115" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L115" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N115" s="12"/>
       <c r="O115" s="1" t="b">
@@ -6376,19 +6369,19 @@
         <v>0.166666666666667</v>
       </c>
       <c r="H116" s="12" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I116" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J116" s="12" t="s">
         <v>21</v>
       </c>
       <c r="K116" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L116" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N116" s="12"/>
       <c r="O116" s="1" t="b">
@@ -6410,68 +6403,68 @@
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="5" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B119" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C119" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D119" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B119" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="C119" s="5" t="s">
+      <c r="E119" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D119" s="5" t="s">
+      <c r="F119" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="E119" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="F119" s="5" t="s">
-        <v>57</v>
-      </c>
       <c r="G119" s="5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H119" s="5" t="s">
         <v>16</v>
       </c>
       <c r="I119" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="J119" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="K119" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="J119" s="5" t="s">
+      <c r="L119" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="K119" s="5" t="s">
+      <c r="M119" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="L119" s="5" t="s">
+      <c r="N119" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="M119" s="5" t="s">
+      <c r="O119" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="N119" s="5" t="s">
+      <c r="P119" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="O119" s="5" t="s">
+      <c r="Q119" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="P119" s="5" t="s">
+      <c r="R119" s="5" t="s">
         <v>83</v>
-      </c>
-      <c r="Q119" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="R119" s="5" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="12" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B120" s="12" t="s">
         <v>1</v>
@@ -6490,22 +6483,22 @@
         <v>0.125</v>
       </c>
       <c r="H120" s="12" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="I120" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J120" s="12" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="K120" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L120" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N120" s="12" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="O120" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -6526,68 +6519,68 @@
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="5" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B123" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C123" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D123" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B123" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="C123" s="5" t="s">
+      <c r="E123" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D123" s="5" t="s">
+      <c r="F123" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="E123" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="F123" s="5" t="s">
-        <v>57</v>
-      </c>
       <c r="G123" s="5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H123" s="5" t="s">
         <v>16</v>
       </c>
       <c r="I123" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="J123" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="K123" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="J123" s="5" t="s">
+      <c r="L123" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="K123" s="5" t="s">
+      <c r="M123" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="L123" s="5" t="s">
+      <c r="N123" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="M123" s="5" t="s">
+      <c r="O123" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="N123" s="5" t="s">
+      <c r="P123" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="O123" s="5" t="s">
+      <c r="Q123" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="P123" s="5" t="s">
+      <c r="R123" s="5" t="s">
         <v>83</v>
-      </c>
-      <c r="Q123" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="R123" s="5" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="12" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B124" s="12" t="s">
         <v>1</v>
@@ -6606,22 +6599,22 @@
         <v>0.0833333333333333</v>
       </c>
       <c r="H124" s="12" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="I124" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J124" s="12" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="K124" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L124" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N124" s="12" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="O124" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -6642,68 +6635,68 @@
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="5" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B127" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C127" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D127" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B127" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="C127" s="5" t="s">
+      <c r="E127" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D127" s="5" t="s">
+      <c r="F127" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="E127" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="F127" s="5" t="s">
-        <v>57</v>
-      </c>
       <c r="G127" s="5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H127" s="5" t="s">
         <v>16</v>
       </c>
       <c r="I127" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="J127" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="K127" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="J127" s="5" t="s">
+      <c r="L127" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="K127" s="5" t="s">
+      <c r="M127" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="L127" s="5" t="s">
+      <c r="N127" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="M127" s="5" t="s">
+      <c r="O127" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="N127" s="5" t="s">
+      <c r="P127" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="O127" s="5" t="s">
+      <c r="Q127" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="P127" s="5" t="s">
+      <c r="R127" s="5" t="s">
         <v>83</v>
-      </c>
-      <c r="Q127" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="R127" s="5" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="12" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B128" s="12" t="s">
         <v>1</v>
@@ -6722,22 +6715,22 @@
         <v>0.125</v>
       </c>
       <c r="H128" s="12" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="I128" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J128" s="12" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="K128" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L128" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N128" s="12" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="O128" s="1" t="b">
         <f aca="false">FALSE()</f>

</xml_diff>